<commit_message>
feat: SMS on bulk fee upload, add phone numbers to 30-student sample, add 4 CE test students file
</commit_message>
<xml_diff>
--- a/backend/excel-files/sample_30_students.xlsx
+++ b/backend/excel-files/sample_30_students.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:H31"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -406,6 +406,7 @@
     <col min="5" max="5" width="40.83203125" customWidth="1"/>
     <col min="6" max="6" width="12.83203125" customWidth="1"/>
     <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,6 +431,9 @@
       <c r="G1" t="str">
         <v>Admission Year</v>
       </c>
+      <c r="H1" t="str">
+        <v>Phone Number</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -453,6 +457,9 @@
       <c r="G2">
         <v>2022</v>
       </c>
+      <c r="H2" t="str">
+        <v>0249690360</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -476,6 +483,9 @@
       <c r="G3">
         <v>2022</v>
       </c>
+      <c r="H3" t="str">
+        <v>0202930167</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -499,6 +509,9 @@
       <c r="G4">
         <v>2022</v>
       </c>
+      <c r="H4" t="str">
+        <v>0271632876</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -522,6 +535,9 @@
       <c r="G5">
         <v>2022</v>
       </c>
+      <c r="H5" t="str">
+        <v>0507143834</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -545,6 +561,9 @@
       <c r="G6">
         <v>2022</v>
       </c>
+      <c r="H6" t="str">
+        <v>0553549073</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -568,6 +587,9 @@
       <c r="G7">
         <v>2022</v>
       </c>
+      <c r="H7" t="str">
+        <v>0277225454</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -591,6 +613,9 @@
       <c r="G8">
         <v>2022</v>
       </c>
+      <c r="H8" t="str">
+        <v>0209533102</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -614,6 +639,9 @@
       <c r="G9">
         <v>2022</v>
       </c>
+      <c r="H9" t="str">
+        <v>0568499196</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -637,6 +665,9 @@
       <c r="G10">
         <v>2024</v>
       </c>
+      <c r="H10" t="str">
+        <v>0201204249</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -660,6 +691,9 @@
       <c r="G11">
         <v>2024</v>
       </c>
+      <c r="H11" t="str">
+        <v>0248555127</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -683,6 +717,9 @@
       <c r="G12">
         <v>2024</v>
       </c>
+      <c r="H12" t="str">
+        <v>0548537748</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -706,6 +743,9 @@
       <c r="G13">
         <v>2024</v>
       </c>
+      <c r="H13" t="str">
+        <v>0597127539</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -729,6 +769,9 @@
       <c r="G14">
         <v>2024</v>
       </c>
+      <c r="H14" t="str">
+        <v>0544263209</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -752,6 +795,9 @@
       <c r="G15">
         <v>2024</v>
       </c>
+      <c r="H15" t="str">
+        <v>0565975654</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -775,6 +821,9 @@
       <c r="G16">
         <v>2024</v>
       </c>
+      <c r="H16" t="str">
+        <v>0561466551</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -798,6 +847,9 @@
       <c r="G17">
         <v>2024</v>
       </c>
+      <c r="H17" t="str">
+        <v>0548554554</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -821,6 +873,9 @@
       <c r="G18">
         <v>2024</v>
       </c>
+      <c r="H18" t="str">
+        <v>0276071602</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -844,6 +899,9 @@
       <c r="G19">
         <v>2024</v>
       </c>
+      <c r="H19" t="str">
+        <v>0245999699</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -867,6 +925,9 @@
       <c r="G20">
         <v>2024</v>
       </c>
+      <c r="H20" t="str">
+        <v>0566286828</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -890,6 +951,9 @@
       <c r="G21">
         <v>2024</v>
       </c>
+      <c r="H21" t="str">
+        <v>0271404331</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
@@ -913,6 +977,9 @@
       <c r="G22">
         <v>2024</v>
       </c>
+      <c r="H22" t="str">
+        <v>0268592825</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
@@ -936,6 +1003,9 @@
       <c r="G23">
         <v>2024</v>
       </c>
+      <c r="H23" t="str">
+        <v>0569365189</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
@@ -959,6 +1029,9 @@
       <c r="G24">
         <v>2024</v>
       </c>
+      <c r="H24" t="str">
+        <v>0245043130</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
@@ -982,6 +1055,9 @@
       <c r="G25">
         <v>2024</v>
       </c>
+      <c r="H25" t="str">
+        <v>0552811767</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
@@ -1005,6 +1081,9 @@
       <c r="G26">
         <v>2024</v>
       </c>
+      <c r="H26" t="str">
+        <v>0279785145</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
@@ -1028,6 +1107,9 @@
       <c r="G27">
         <v>2024</v>
       </c>
+      <c r="H27" t="str">
+        <v>0572392503</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
@@ -1051,6 +1133,9 @@
       <c r="G28">
         <v>2024</v>
       </c>
+      <c r="H28" t="str">
+        <v>0244213382</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
@@ -1074,6 +1159,9 @@
       <c r="G29">
         <v>2024</v>
       </c>
+      <c r="H29" t="str">
+        <v>0598647284</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
@@ -1097,6 +1185,9 @@
       <c r="G30">
         <v>2024</v>
       </c>
+      <c r="H30" t="str">
+        <v>0502089697</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
@@ -1120,10 +1211,13 @@
       <c r="G31">
         <v>2024</v>
       </c>
+      <c r="H31" t="str">
+        <v>0563190772</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H31"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>